<commit_message>
feat: co-author import support, ResearchPolicy can_edit fix, import tests 25/25
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/tests/e2e/fixtures/research_import_duplicate.xlsx
+++ b/tests/e2e/fixtures/research_import_duplicate.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O3"/>
+  <dimension ref="A1:Q3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -445,6 +445,12 @@
       <c r="O1" t="str">
         <v>is_scopus_indexed</v>
       </c>
+      <c r="P1" t="str">
+        <v>coauthor_emails</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>coauthor_can_edit</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -492,6 +498,12 @@
       <c r="O2" t="str">
         <v>OPTIONAL. 0|1</v>
       </c>
+      <c r="P2" t="str">
+        <v>OPTIONAL. Pipe-separated co-author emails</v>
+      </c>
+      <c r="Q2" t="str">
+        <v>OPTIONAL. Pipe-separated 0|1 matching coauthors (default 1)</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -539,10 +551,16 @@
       <c r="O3">
         <v>1</v>
       </c>
+      <c r="P3" t="str">
+        <v/>
+      </c>
+      <c r="Q3" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
test: full suite 205/205 passing — program_code, document_url, all import tests verified
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/tests/e2e/fixtures/research_import_duplicate.xlsx
+++ b/tests/e2e/fixtures/research_import_duplicate.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q3"/>
+  <dimension ref="A1:S3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -451,6 +451,12 @@
       <c r="Q1" t="str">
         <v>coauthor_can_edit</v>
       </c>
+      <c r="R1" t="str">
+        <v>document_url</v>
+      </c>
+      <c r="S1" t="str">
+        <v>document_label</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -504,6 +510,12 @@
       <c r="Q2" t="str">
         <v>OPTIONAL. Pipe-separated 0|1 matching coauthors (default 1)</v>
       </c>
+      <c r="R2" t="str">
+        <v>OPTIONAL. Pipe-separated https:// URLs</v>
+      </c>
+      <c r="S2" t="str">
+        <v>OPTIONAL. Pipe-separated labels matching document_url</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -557,10 +569,16 @@
       <c r="Q3" t="str">
         <v/>
       </c>
+      <c r="R3" t="str">
+        <v/>
+      </c>
+      <c r="S3" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Q3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>